<commit_message>
chore(fem): re-save griffiths1_load input from Studio
In-place re-save of the input workbook (sidecar reconciliation on save).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fem/files/xslope_griffiths1_load.xlsx
+++ b/docs/fem/files/xslope_griffiths1_load.xlsx
@@ -37,7 +37,7 @@
     <definedName name="solution2">mat!#REF!</definedName>
     <definedName name="version">main!$D$5</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -8000,7 +8000,7 @@
         <v>49</v>
       </c>
       <c r="D9" s="1">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>19</v>
@@ -8014,7 +8014,7 @@
         <v>48</v>
       </c>
       <c r="D10" s="1">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>17</v>
@@ -8029,7 +8029,7 @@
         <v>75</v>
       </c>
       <c r="D11" s="1">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>21</v>
@@ -9460,40 +9460,73 @@
       <c r="A9" s="3">
         <v>1</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>153</v>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>soil</t>
+        </is>
       </c>
       <c r="C9" s="3">
-        <v>125</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>67</v>
+        <v>125.0</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>mc</t>
+        </is>
       </c>
       <c r="E9" s="3">
-        <f>C9*50*0.05</f>
         <v>312.5</v>
       </c>
       <c r="F9" s="3">
-        <v>20</v>
-      </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
+        <v>20.0</v>
+      </c>
+      <c r="G9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="I9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J9" s="3">
+        <v>0.0</v>
+      </c>
       <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="3"/>
-      <c r="P9" s="3"/>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="3"/>
-      <c r="S9" s="3"/>
-      <c r="T9" s="3"/>
-      <c r="U9" s="3"/>
-      <c r="V9" s="3"/>
+      <c r="L9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="M9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="N9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="O9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="P9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="Q9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="R9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="S9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="T9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="U9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="V9" s="3">
+        <v>0.0</v>
+      </c>
       <c r="W9" s="43">
-        <v>700000</v>
+        <v>700000.0</v>
       </c>
       <c r="X9" s="3">
         <v>0.3</v>
@@ -10249,15 +10282,17 @@
         <v>46</v>
       </c>
       <c r="B2" s="3">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="D2" s="27" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="46" t="s">
-        <v>2</v>
+      <c r="A4" s="46" t="inlineStr">
+        <is>
+          <t>Profile Line #1</t>
+        </is>
       </c>
       <c r="B4" s="46"/>
       <c r="D4" s="46" t="s">
@@ -10612,10 +10647,10 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="B8" s="3">
-        <v>50</v>
+        <v>50.0</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
@@ -10656,11 +10691,10 @@
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
-        <f>1.2*B8</f>
-        <v>60</v>
+        <v>60.0</v>
       </c>
       <c r="B9" s="3">
-        <v>50</v>
+        <v>50.0</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -10701,11 +10735,10 @@
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
-        <f>A9+2*B8</f>
-        <v>160</v>
+        <v>160.0</v>
       </c>
       <c r="B10" s="3">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
@@ -11673,16 +11706,18 @@
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>120</v>
+        <v>120.0</v>
       </c>
       <c r="C3" s="3">
-        <v>80</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>26</v>
+        <v>80.0</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Depth</t>
+        </is>
       </c>
       <c r="E3" s="3">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -12114,13 +12149,13 @@
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B4" s="3">
-        <v>30</v>
+        <v>30.0</v>
       </c>
       <c r="C4" s="3">
-        <v>50</v>
+        <v>50.0</v>
       </c>
       <c r="D4" s="3">
-        <v>800</v>
+        <v>800.0</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -12140,13 +12175,13 @@
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="3">
-        <v>45</v>
+        <v>45.0</v>
       </c>
       <c r="C5" s="3">
-        <v>50</v>
+        <v>50.0</v>
       </c>
       <c r="D5" s="3">
-        <v>800</v>
+        <v>800.0</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>

</xml_diff>